<commit_message>
change level of some messages
fixes issue #224
</commit_message>
<xml_diff>
--- a/RiseClipseValidatorSCLMessages.xlsx
+++ b/RiseClipseValidatorSCLMessages.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcadet/git/RiseClipse/GitHub/riseclipse-validator-scl2003/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EAEFB5F-63E9-094F-A2DB-E9783CD56887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6712483E-75E1-704B-A403-2F4F98969A1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="620" yWindow="660" windowWidth="36300" windowHeight="27680" xr2:uid="{D58BF774-7A59-3C48-B3D5-ECB80F73968C}"/>
+    <workbookView xWindow="51200" yWindow="640" windowWidth="36300" windowHeight="27680" xr2:uid="{D58BF774-7A59-3C48-B3D5-ECB80F73968C}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$C$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$C$113</definedName>
   </definedNames>
   <calcPr calcId="181029" iterateDelta="1E-4"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="144">
   <si>
     <t>NSD/Validation</t>
   </si>
@@ -468,6 +468,9 @@
   </si>
   <si>
     <t>Message</t>
+  </si>
+  <si>
+    <t>NOTICE</t>
   </si>
 </sst>
 </file>
@@ -900,24 +903,24 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="B5" t="s">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>8</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -928,7 +931,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -939,7 +942,7 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -950,29 +953,29 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B10" t="s">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B11" t="s">
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -983,7 +986,7 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -994,7 +997,7 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -1005,29 +1008,29 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B16" t="s">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -1038,7 +1041,7 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>13</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -1049,7 +1052,7 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>15</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -1060,7 +1063,7 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -1071,7 +1074,7 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -1082,7 +1085,7 @@
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -1093,7 +1096,7 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -1104,7 +1107,7 @@
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -1115,7 +1118,7 @@
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>78</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -1126,7 +1129,7 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>79</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
@@ -1137,7 +1140,7 @@
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -1148,7 +1151,7 @@
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
@@ -1159,7 +1162,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>59</v>
+        <v>80</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -1170,7 +1173,7 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>60</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -1181,7 +1184,7 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -1192,7 +1195,7 @@
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
@@ -1203,7 +1206,7 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -1214,7 +1217,7 @@
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -1225,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -1236,7 +1239,7 @@
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -1247,29 +1250,29 @@
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="B37" t="s">
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>21</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="B38" t="s">
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>22</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -1280,7 +1283,7 @@
         <v>1</v>
       </c>
       <c r="C39" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -1291,7 +1294,7 @@
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -1302,7 +1305,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -1313,7 +1316,7 @@
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -1324,7 +1327,7 @@
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -1335,7 +1338,7 @@
         <v>1</v>
       </c>
       <c r="C44" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -1346,7 +1349,7 @@
         <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
@@ -1357,7 +1360,7 @@
         <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -1368,7 +1371,7 @@
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
@@ -1379,7 +1382,7 @@
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
@@ -1390,7 +1393,7 @@
         <v>1</v>
       </c>
       <c r="C49" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
@@ -1401,7 +1404,7 @@
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -1412,7 +1415,7 @@
         <v>1</v>
       </c>
       <c r="C51" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
@@ -1423,7 +1426,7 @@
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
@@ -1434,7 +1437,7 @@
         <v>1</v>
       </c>
       <c r="C53" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -1445,7 +1448,7 @@
         <v>1</v>
       </c>
       <c r="C54" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
@@ -1456,7 +1459,7 @@
         <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
@@ -1467,7 +1470,7 @@
         <v>1</v>
       </c>
       <c r="C56" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
@@ -1478,7 +1481,7 @@
         <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
@@ -1489,7 +1492,7 @@
         <v>1</v>
       </c>
       <c r="C58" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
@@ -1500,7 +1503,7 @@
         <v>1</v>
       </c>
       <c r="C59" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
@@ -1511,29 +1514,29 @@
         <v>1</v>
       </c>
       <c r="C60" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B61" t="s">
         <v>1</v>
       </c>
       <c r="C61" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B62" t="s">
         <v>1</v>
       </c>
       <c r="C62" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
@@ -1544,7 +1547,7 @@
         <v>1</v>
       </c>
       <c r="C63" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
@@ -1555,51 +1558,51 @@
         <v>1</v>
       </c>
       <c r="C64" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B65" t="s">
         <v>1</v>
       </c>
       <c r="C65" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="B66" t="s">
         <v>1</v>
       </c>
       <c r="C66" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="B67" t="s">
         <v>1</v>
       </c>
       <c r="C67" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>86</v>
+        <v>5</v>
       </c>
       <c r="B68" t="s">
         <v>1</v>
       </c>
       <c r="C68" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
@@ -1610,7 +1613,7 @@
         <v>1</v>
       </c>
       <c r="C69" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
@@ -1621,7 +1624,7 @@
         <v>1</v>
       </c>
       <c r="C70" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -1632,7 +1635,7 @@
         <v>1</v>
       </c>
       <c r="C71" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
@@ -1643,7 +1646,7 @@
         <v>1</v>
       </c>
       <c r="C72" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
@@ -1654,7 +1657,7 @@
         <v>1</v>
       </c>
       <c r="C73" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
@@ -1665,7 +1668,7 @@
         <v>1</v>
       </c>
       <c r="C74" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
@@ -1676,7 +1679,7 @@
         <v>1</v>
       </c>
       <c r="C75" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
@@ -1687,7 +1690,7 @@
         <v>1</v>
       </c>
       <c r="C76" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
@@ -1698,7 +1701,7 @@
         <v>1</v>
       </c>
       <c r="C77" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
@@ -1709,40 +1712,40 @@
         <v>1</v>
       </c>
       <c r="C78" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="B79" t="s">
         <v>1</v>
       </c>
       <c r="C79" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="B80" t="s">
         <v>1</v>
       </c>
       <c r="C80" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="B81" t="s">
         <v>1</v>
       </c>
       <c r="C81" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
@@ -1753,7 +1756,7 @@
         <v>1</v>
       </c>
       <c r="C82" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
@@ -1764,7 +1767,7 @@
         <v>1</v>
       </c>
       <c r="C83" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
@@ -1775,7 +1778,7 @@
         <v>1</v>
       </c>
       <c r="C84" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
@@ -1786,7 +1789,7 @@
         <v>1</v>
       </c>
       <c r="C85" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
@@ -1797,7 +1800,7 @@
         <v>1</v>
       </c>
       <c r="C86" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
@@ -1808,7 +1811,7 @@
         <v>1</v>
       </c>
       <c r="C87" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
@@ -1819,7 +1822,7 @@
         <v>1</v>
       </c>
       <c r="C88" t="s">
-        <v>91</v>
+        <v>61</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
@@ -1830,7 +1833,7 @@
         <v>1</v>
       </c>
       <c r="C89" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
@@ -1841,7 +1844,7 @@
         <v>1</v>
       </c>
       <c r="C90" t="s">
-        <v>93</v>
+        <v>63</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
@@ -1852,7 +1855,7 @@
         <v>1</v>
       </c>
       <c r="C91" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
@@ -1863,51 +1866,51 @@
         <v>1</v>
       </c>
       <c r="C92" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="B93" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C93" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="B94" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C94" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="B95" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C95" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B96" t="s">
         <v>4</v>
       </c>
       <c r="C96" t="s">
-        <v>3</v>
+        <v>134</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
@@ -1918,7 +1921,7 @@
         <v>4</v>
       </c>
       <c r="C97" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
@@ -1929,216 +1932,216 @@
         <v>4</v>
       </c>
       <c r="C98" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>12</v>
+        <v>130</v>
       </c>
       <c r="B99" t="s">
         <v>4</v>
       </c>
       <c r="C99" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>12</v>
+        <v>130</v>
       </c>
       <c r="B100" t="s">
         <v>4</v>
       </c>
       <c r="C100" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>12</v>
+        <v>130</v>
       </c>
       <c r="B101" t="s">
         <v>4</v>
       </c>
       <c r="C101" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B102" t="s">
         <v>4</v>
       </c>
       <c r="C102" t="s">
-        <v>135</v>
+        <v>106</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="B103" t="s">
         <v>4</v>
       </c>
       <c r="C103" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>130</v>
+        <v>45</v>
       </c>
       <c r="B104" t="s">
         <v>4</v>
       </c>
       <c r="C104" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>130</v>
+        <v>5</v>
       </c>
       <c r="B105" t="s">
         <v>4</v>
       </c>
       <c r="C105" t="s">
-        <v>139</v>
+        <v>105</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="B106" t="s">
         <v>4</v>
       </c>
       <c r="C106" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="B107" t="s">
         <v>4</v>
       </c>
       <c r="C107" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="B108" t="s">
         <v>4</v>
       </c>
       <c r="C108" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="B109" t="s">
         <v>4</v>
       </c>
       <c r="C109" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="B110" t="s">
         <v>4</v>
       </c>
       <c r="C110" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="B111" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C111" t="s">
-        <v>112</v>
+        <v>3</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="B112" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C112" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="B113" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C113" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="B114" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C114" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="B115" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C115" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="B116" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C116" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B117" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C117" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
@@ -2146,10 +2149,10 @@
         <v>45</v>
       </c>
       <c r="B118" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C118" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
@@ -2157,10 +2160,10 @@
         <v>45</v>
       </c>
       <c r="B119" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C119" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
@@ -2168,10 +2171,10 @@
         <v>45</v>
       </c>
       <c r="B120" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C120" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.2">
@@ -2179,10 +2182,10 @@
         <v>45</v>
       </c>
       <c r="B121" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C121" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
@@ -2190,10 +2193,10 @@
         <v>45</v>
       </c>
       <c r="B122" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C122" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
@@ -2201,10 +2204,10 @@
         <v>45</v>
       </c>
       <c r="B123" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C123" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
@@ -2212,10 +2215,10 @@
         <v>45</v>
       </c>
       <c r="B124" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C124" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
@@ -2223,10 +2226,10 @@
         <v>45</v>
       </c>
       <c r="B125" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C125" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
@@ -2234,10 +2237,10 @@
         <v>45</v>
       </c>
       <c r="B126" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C126" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.2">
@@ -2245,104 +2248,104 @@
         <v>45</v>
       </c>
       <c r="B127" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C127" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B128" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C128" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="B129" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C129" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="B130" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C130" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>86</v>
+        <v>45</v>
       </c>
       <c r="B131" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C131" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="B132" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C132" t="s">
-        <v>97</v>
+        <v>123</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="B133" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C133" t="s">
-        <v>98</v>
+        <v>124</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="B134" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C134" t="s">
-        <v>99</v>
+        <v>125</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="B135" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="C135" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C137" xr:uid="{98F32A72-AC13-4647-A6BC-C931315F0D46}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C137">
-      <sortCondition ref="B1:B137"/>
+  <autoFilter ref="A1:C113" xr:uid="{98F32A72-AC13-4647-A6BC-C931315F0D46}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C113">
+      <sortCondition ref="B1:B113"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>